<commit_message>
Strategies added, responsives assigned
</commit_message>
<xml_diff>
--- a/docs/src/Morze_Risks.xlsx
+++ b/docs/src/Morze_Risks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE4D7DB-D2D7-4D24-9098-5626B09B9527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F380DD5-87E5-439B-80C2-7B4F738D76AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Таблица задач" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="243">
   <si>
     <t>Ид.</t>
   </si>
@@ -522,9 +522,6 @@
     <t>Сократить объем 1-й итерации, принять временное решение</t>
   </si>
   <si>
-    <t>Тимлид</t>
-  </si>
-  <si>
     <t>Открыт</t>
   </si>
   <si>
@@ -543,9 +540,6 @@
     <t>Вести задачи временно в Excel/Notion</t>
   </si>
   <si>
-    <t>PM / DevOps</t>
-  </si>
-  <si>
     <t>R3</t>
   </si>
   <si>
@@ -564,9 +558,6 @@
     <t>Переделка схемы с миграциями, заморозка API</t>
   </si>
   <si>
-    <t>Backend</t>
-  </si>
-  <si>
     <t>R4</t>
   </si>
   <si>
@@ -585,9 +576,6 @@
     <t>Перенести второстепенные сценарии в backlog</t>
   </si>
   <si>
-    <t>Analyst / Frontend</t>
-  </si>
-  <si>
     <t>R5</t>
   </si>
   <si>
@@ -603,9 +591,6 @@
     <t>Делать технический UI без финального дизайна</t>
   </si>
   <si>
-    <t>Frontend / Designer</t>
-  </si>
-  <si>
     <t>R6</t>
   </si>
   <si>
@@ -624,9 +609,6 @@
     <t>Срочный hotfix API/adapter-слой</t>
   </si>
   <si>
-    <t>Backend + Frontend</t>
-  </si>
-  <si>
     <t>Критичный</t>
   </si>
   <si>
@@ -645,9 +627,6 @@
     <t>Резерв 2–3 дня на исправления</t>
   </si>
   <si>
-    <t>QA / Team</t>
-  </si>
-  <si>
     <t>R8</t>
   </si>
   <si>
@@ -663,9 +642,6 @@
     <t>Сфокусироваться на критических сценариях</t>
   </si>
   <si>
-    <t>QA</t>
-  </si>
-  <si>
     <t>R9</t>
   </si>
   <si>
@@ -681,9 +657,6 @@
     <t>Выделить отдельный день на финальную сборку документации</t>
   </si>
   <si>
-    <t>PM / Analyst</t>
-  </si>
-  <si>
     <t>R10</t>
   </si>
   <si>
@@ -702,9 +675,6 @@
     <t>Исключить низкоприоритетные функции</t>
   </si>
   <si>
-    <t>Заказчик / PM</t>
-  </si>
-  <si>
     <t>R11</t>
   </si>
   <si>
@@ -738,9 +708,6 @@
     <t>Сократить нефункциональные доработки</t>
   </si>
   <si>
-    <t>PM</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
@@ -778,6 +745,33 @@
   </si>
   <si>
     <t>Morze</t>
+  </si>
+  <si>
+    <t>Стратегия</t>
+  </si>
+  <si>
+    <t>Избежание</t>
+  </si>
+  <si>
+    <t>Снижение</t>
+  </si>
+  <si>
+    <t>Парфенов А.</t>
+  </si>
+  <si>
+    <t>Гареев Г.</t>
+  </si>
+  <si>
+    <t>Бугаков И.</t>
+  </si>
+  <si>
+    <t>Парфенов А., Гареев Г.</t>
+  </si>
+  <si>
+    <t>Парфенов А., Гареев Г., Бугаков И.</t>
+  </si>
+  <si>
+    <t>Гареев Г., Бугаков И.</t>
   </si>
 </sst>
 </file>
@@ -785,21 +779,29 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="8">
-    <numFmt numFmtId="169" formatCode="&quot;R9&quot;"/>
-    <numFmt numFmtId="170" formatCode="&quot;&quot;"/>
-    <numFmt numFmtId="171" formatCode="&quot;R5&quot;"/>
-    <numFmt numFmtId="172" formatCode="&quot;R6&quot;"/>
-    <numFmt numFmtId="174" formatCode="&quot;R4, R8, R11&quot;"/>
-    <numFmt numFmtId="175" formatCode="&quot;R1, R3, R7, R10&quot;"/>
-    <numFmt numFmtId="176" formatCode="&quot;R12&quot;"/>
-    <numFmt numFmtId="177" formatCode="&quot;&quot;\R\2&quot;&quot;"/>
+    <numFmt numFmtId="164" formatCode="&quot;R9&quot;"/>
+    <numFmt numFmtId="165" formatCode="&quot;&quot;"/>
+    <numFmt numFmtId="166" formatCode="&quot;R5&quot;"/>
+    <numFmt numFmtId="167" formatCode="&quot;R6&quot;"/>
+    <numFmt numFmtId="168" formatCode="&quot;R4, R8, R11&quot;"/>
+    <numFmt numFmtId="169" formatCode="&quot;R1, R3, R7, R10&quot;"/>
+    <numFmt numFmtId="170" formatCode="&quot;R12&quot;"/>
+    <numFmt numFmtId="171" formatCode="&quot;&quot;\R\2&quot;&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -840,12 +842,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -854,31 +856,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -896,7 +898,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1265,7 +1273,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -2503,12 +2511,16 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EA9BC20-6F7E-4B17-89CC-040ED8288612}">
-  <dimension ref="A1:N13"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" bestFit="1" customWidth="1"/>
@@ -2518,13 +2530,14 @@
     <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.44140625" customWidth="1"/>
     <col min="7" max="7" width="22.44140625" customWidth="1"/>
-    <col min="8" max="8" width="20.21875" customWidth="1"/>
-    <col min="9" max="9" width="25.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.88671875" customWidth="1"/>
-    <col min="11" max="11" width="10.33203125" customWidth="1"/>
+    <col min="8" max="8" width="24.88671875" customWidth="1"/>
+    <col min="9" max="9" width="27.5546875" customWidth="1"/>
+    <col min="10" max="10" width="12.88671875" style="17" customWidth="1"/>
+    <col min="11" max="11" width="21.33203125" customWidth="1"/>
+    <col min="12" max="12" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>143</v>
       </c>
@@ -2547,19 +2560,26 @@
         <v>149</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="J1" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+    </row>
+    <row r="2" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>154</v>
       </c>
@@ -2583,24 +2603,31 @@
         <v>156</v>
       </c>
       <c r="H2" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="20"/>
+      <c r="R2" s="3"/>
+    </row>
+    <row r="3" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>161</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>162</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>50</v>
@@ -2616,30 +2643,37 @@
         <v>6</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>164</v>
       </c>
       <c r="I3" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="J3" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="20"/>
+      <c r="R3" s="3"/>
+    </row>
+    <row r="4" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="B4" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>167</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>169</v>
       </c>
       <c r="D4" s="1">
         <v>3</v>
@@ -2652,33 +2686,40 @@
         <v>15</v>
       </c>
       <c r="G4" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="I4" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="J4" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="N4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="3"/>
+    </row>
+    <row r="5" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>173</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="N4" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>176</v>
       </c>
       <c r="D5" s="1">
         <v>3</v>
@@ -2691,27 +2732,34 @@
         <v>12</v>
       </c>
       <c r="G5" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J5" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="3"/>
+    </row>
+    <row r="6" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="B6" s="4" t="s">
         <v>178</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>182</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>74</v>
@@ -2727,30 +2775,37 @@
         <v>16</v>
       </c>
       <c r="G6" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="J6" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="3"/>
+    </row>
+    <row r="7" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>184</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>189</v>
       </c>
       <c r="D7" s="1">
         <v>4</v>
@@ -2763,27 +2818,34 @@
         <v>20</v>
       </c>
       <c r="G7" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="J7" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="20"/>
+      <c r="R7" s="3"/>
+    </row>
+    <row r="8" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>190</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>196</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>135</v>
@@ -2799,27 +2861,34 @@
         <v>15</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>192</v>
+      </c>
+      <c r="J8" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="20"/>
+      <c r="R8" s="3"/>
+    </row>
+    <row r="9" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>119</v>
@@ -2835,27 +2904,34 @@
         <v>12</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+      <c r="J9" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="20"/>
+      <c r="R9" s="3"/>
+    </row>
+    <row r="10" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>81</v>
@@ -2871,30 +2947,37 @@
         <v>12</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+      <c r="J10" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="20"/>
+      <c r="R10" s="3"/>
+    </row>
+    <row r="11" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="D11" s="1">
         <v>3</v>
@@ -2907,27 +2990,34 @@
         <v>15</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="J11" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="20"/>
+      <c r="R11" s="3"/>
+    </row>
+    <row r="12" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>101</v>
@@ -2943,30 +3033,37 @@
         <v>12</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>213</v>
+      </c>
+      <c r="J12" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="Q12" s="20"/>
+      <c r="R12" s="3"/>
+    </row>
+    <row r="13" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="D13" s="1">
         <v>2</v>
@@ -2979,34 +3076,38 @@
         <v>10</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>160</v>
-      </c>
+        <v>219</v>
+      </c>
+      <c r="J13" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="20"/>
+      <c r="R13" s="3"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="K14" s="4"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="K16" s="4"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F14:F18">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="F2:F13">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -3029,13 +3130,28 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <conditionalFormatting sqref="F14:F18">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="60" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C20C0C9-F97B-4C1D-942F-BAC2702ABDB2}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3044,27 +3160,27 @@
   <sheetData>
     <row r="1" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="B2" s="5">
         <v>5</v>
@@ -3084,7 +3200,7 @@
     </row>
     <row r="3" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="B3" s="5">
         <v>4</v>
@@ -3107,7 +3223,7 @@
     </row>
     <row r="4" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="B4" s="5">
         <v>3</v>
@@ -3130,7 +3246,7 @@
     </row>
     <row r="5" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="B5" s="5">
         <v>2</v>
@@ -3153,7 +3269,7 @@
     </row>
     <row r="6" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="B6" s="5">
         <v>1</v>
@@ -3196,6 +3312,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>